<commit_message>
Migrate UI from Streamlit to React; add dashboard analytics, filled map interactions, and README update
Includes frontend Vite app, FastAPI-backed dashboard enhancements, choropleth market map with slicer-driven selection, and updated project documentation.
</commit_message>
<xml_diff>
--- a/data/Complete-DB.xlsx
+++ b/data/Complete-DB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\70091424\Downloads\Trial3\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1BE01E-FAC6-43F5-B9D6-3C395A7800B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C638699C-AA6D-4B7D-9A39-7E16A9569924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="All Projects" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Projects'!$F$1:$F$814</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Projects'!$D$1:$D$814</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4756" uniqueCount="964">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4756" uniqueCount="963">
   <si>
     <t>Category</t>
   </si>
@@ -2483,9 +2483,6 @@
   </si>
   <si>
     <t>AB InBev Jupiler</t>
-  </si>
-  <si>
-    <t>First Abu DhAB InBev Bank</t>
   </si>
   <si>
     <t>TCPL Gold</t>
@@ -3386,25 +3383,25 @@
   <sheetData>
     <row r="1" spans="1:8" s="2" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>961</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>960</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>962</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>961</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>963</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3541,7 +3538,7 @@
         <v>12</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>13</v>
@@ -3564,7 +3561,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>13</v>
@@ -3722,7 +3719,7 @@
         <v>12</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>24</v>
@@ -3808,7 +3805,7 @@
         <v>28</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>29</v>
@@ -3831,13 +3828,13 @@
         <v>28</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>30</v>
@@ -4090,7 +4087,7 @@
         <v>45</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>4</v>
@@ -4205,7 +4202,7 @@
         <v>52</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>53</v>
@@ -4251,7 +4248,7 @@
         <v>55</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>40</v>
@@ -4274,7 +4271,7 @@
         <v>55</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>40</v>
@@ -4300,7 +4297,7 @@
         <v>57</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>7</v>
@@ -4323,7 +4320,7 @@
         <v>58</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>7</v>
@@ -4386,7 +4383,7 @@
         <v>403</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>64</v>
@@ -4430,10 +4427,10 @@
         <v>403</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>66</v>
@@ -4453,10 +4450,10 @@
         <v>403</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>66</v>
@@ -4476,10 +4473,10 @@
         <v>403</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>66</v>
@@ -4499,7 +4496,7 @@
         <v>403</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>67</v>
@@ -4522,10 +4519,10 @@
         <v>403</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>66</v>
@@ -4545,7 +4542,7 @@
         <v>403</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>68</v>
@@ -4568,10 +4565,10 @@
         <v>403</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>66</v>
@@ -4591,10 +4588,10 @@
         <v>403</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>66</v>
@@ -4784,7 +4781,7 @@
         <v>48</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -4864,7 +4861,7 @@
         <v>77</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>85</v>
@@ -5002,7 +4999,7 @@
         <v>77</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>92</v>
@@ -5025,7 +5022,7 @@
         <v>77</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>94</v>
@@ -5048,7 +5045,7 @@
         <v>77</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>94</v>
@@ -5071,13 +5068,13 @@
         <v>77</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>94</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="F74" s="9" t="s">
         <v>4</v>
@@ -5347,7 +5344,7 @@
         <v>112</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>113</v>
@@ -5370,7 +5367,7 @@
         <v>112</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>113</v>
@@ -5393,7 +5390,7 @@
         <v>112</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>113</v>
@@ -5627,7 +5624,7 @@
         <v>762</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="F98" s="9" t="s">
         <v>30</v>
@@ -5725,7 +5722,7 @@
         <v>66</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -5782,7 +5779,7 @@
         <v>112</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>141</v>
@@ -5805,13 +5802,13 @@
         <v>112</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>141</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="F106" s="9" t="s">
         <v>40</v>
@@ -5828,7 +5825,7 @@
         <v>28</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>143</v>
@@ -5851,7 +5848,7 @@
         <v>28</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>146</v>
@@ -5880,7 +5877,7 @@
         <v>149</v>
       </c>
       <c r="E109" s="3" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="F109" s="9" t="s">
         <v>30</v>
@@ -5903,7 +5900,7 @@
         <v>149</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F110" s="9" t="s">
         <v>30</v>
@@ -5920,7 +5917,7 @@
         <v>28</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>150</v>
@@ -5943,7 +5940,7 @@
         <v>28</v>
       </c>
       <c r="C112" s="7" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>152</v>
@@ -5966,7 +5963,7 @@
         <v>28</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>152</v>
@@ -5989,7 +5986,7 @@
         <v>28</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>152</v>
@@ -6012,7 +6009,7 @@
         <v>28</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>152</v>
@@ -6035,7 +6032,7 @@
         <v>28</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>152</v>
@@ -6058,7 +6055,7 @@
         <v>28</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>152</v>
@@ -6081,7 +6078,7 @@
         <v>28</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>159</v>
@@ -6162,7 +6159,7 @@
         <v>66</v>
       </c>
       <c r="G121" s="9" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -6182,7 +6179,7 @@
         <v>163</v>
       </c>
       <c r="F122" s="9" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="G122" s="9" t="s">
         <v>5</v>
@@ -6208,7 +6205,7 @@
         <v>90</v>
       </c>
       <c r="G123" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -6225,13 +6222,13 @@
         <v>164</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="F124" s="9" t="s">
         <v>90</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -6265,7 +6262,7 @@
         <v>2</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>791</v>
@@ -6288,7 +6285,7 @@
         <v>112</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>167</v>
@@ -6317,7 +6314,7 @@
         <v>168</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="F128" s="9" t="s">
         <v>169</v>
@@ -6337,7 +6334,7 @@
         <v>799</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E129" s="3" t="s">
         <v>168</v>
@@ -6360,7 +6357,7 @@
         <v>799</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E130" s="3" t="s">
         <v>168</v>
@@ -6383,7 +6380,7 @@
         <v>799</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E131" s="3" t="s">
         <v>168</v>
@@ -6406,7 +6403,7 @@
         <v>799</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E132" s="3" t="s">
         <v>168</v>
@@ -6429,7 +6426,7 @@
         <v>799</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E133" s="3" t="s">
         <v>168</v>
@@ -6452,7 +6449,7 @@
         <v>799</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E134" s="3" t="s">
         <v>168</v>
@@ -6475,13 +6472,13 @@
         <v>799</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E135" s="3" t="s">
         <v>168</v>
       </c>
       <c r="F135" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G135" s="9" t="s">
         <v>170</v>
@@ -6498,7 +6495,7 @@
         <v>799</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E136" s="3" t="s">
         <v>168</v>
@@ -6521,7 +6518,7 @@
         <v>799</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E137" s="3" t="s">
         <v>168</v>
@@ -6544,7 +6541,7 @@
         <v>799</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E138" s="3" t="s">
         <v>168</v>
@@ -6567,7 +6564,7 @@
         <v>799</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E139" s="3" t="s">
         <v>168</v>
@@ -6590,7 +6587,7 @@
         <v>799</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E140" s="3" t="s">
         <v>168</v>
@@ -6639,7 +6636,7 @@
         <v>175</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="F142" s="9" t="s">
         <v>90</v>
@@ -6656,7 +6653,7 @@
         <v>2</v>
       </c>
       <c r="C143" s="7" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>791</v>
@@ -6866,7 +6863,7 @@
         <v>186</v>
       </c>
       <c r="F152" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G152" s="9" t="s">
         <v>183</v>
@@ -6889,7 +6886,7 @@
         <v>187</v>
       </c>
       <c r="F153" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G153" s="9" t="s">
         <v>183</v>
@@ -7004,7 +7001,7 @@
         <v>187</v>
       </c>
       <c r="F158" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G158" s="9" t="s">
         <v>190</v>
@@ -7027,7 +7024,7 @@
         <v>189</v>
       </c>
       <c r="F159" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G159" s="9" t="s">
         <v>190</v>
@@ -7050,7 +7047,7 @@
         <v>188</v>
       </c>
       <c r="F160" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G160" s="9" t="s">
         <v>190</v>
@@ -7073,7 +7070,7 @@
         <v>185</v>
       </c>
       <c r="F161" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G161" s="9" t="s">
         <v>190</v>
@@ -7096,7 +7093,7 @@
         <v>192</v>
       </c>
       <c r="F162" s="9" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G162" s="9"/>
     </row>
@@ -7117,7 +7114,7 @@
         <v>193</v>
       </c>
       <c r="F163" s="9" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G163" s="9"/>
     </row>
@@ -7135,7 +7132,7 @@
         <v>194</v>
       </c>
       <c r="E164" s="6" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="F164" s="9" t="s">
         <v>325</v>
@@ -7180,7 +7177,7 @@
         <v>196</v>
       </c>
       <c r="F166" s="9" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="G166" s="9" t="s">
         <v>183</v>
@@ -7203,7 +7200,7 @@
         <v>196</v>
       </c>
       <c r="F167" s="9" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="G167" s="9" t="s">
         <v>183</v>
@@ -7226,7 +7223,7 @@
         <v>196</v>
       </c>
       <c r="F168" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G168" s="9" t="s">
         <v>190</v>
@@ -7249,7 +7246,7 @@
         <v>196</v>
       </c>
       <c r="F169" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G169" s="9" t="s">
         <v>190</v>
@@ -7272,7 +7269,7 @@
         <v>180</v>
       </c>
       <c r="F170" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G170" s="9" t="s">
         <v>145</v>
@@ -7295,7 +7292,7 @@
         <v>198</v>
       </c>
       <c r="F171" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G171" s="9" t="s">
         <v>145</v>
@@ -7318,7 +7315,7 @@
         <v>199</v>
       </c>
       <c r="F172" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G172" s="9" t="s">
         <v>190</v>
@@ -7341,7 +7338,7 @@
         <v>200</v>
       </c>
       <c r="F173" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G173" s="9" t="s">
         <v>190</v>
@@ -7364,7 +7361,7 @@
         <v>201</v>
       </c>
       <c r="F174" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G174" s="9" t="s">
         <v>190</v>
@@ -7387,7 +7384,7 @@
         <v>202</v>
       </c>
       <c r="F175" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G175" s="9" t="s">
         <v>190</v>
@@ -7410,7 +7407,7 @@
         <v>203</v>
       </c>
       <c r="F176" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G176" s="9" t="s">
         <v>183</v>
@@ -7433,7 +7430,7 @@
         <v>204</v>
       </c>
       <c r="F177" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G177" s="9"/>
     </row>
@@ -7454,7 +7451,7 @@
         <v>198</v>
       </c>
       <c r="F178" s="9" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="G178" s="9" t="s">
         <v>145</v>
@@ -7477,7 +7474,7 @@
         <v>814</v>
       </c>
       <c r="F179" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G179" s="9" t="s">
         <v>38</v>
@@ -7500,7 +7497,7 @@
         <v>206</v>
       </c>
       <c r="F180" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G180" s="9" t="s">
         <v>38</v>
@@ -7523,7 +7520,7 @@
         <v>12</v>
       </c>
       <c r="F181" s="9" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="G181" s="9" t="s">
         <v>7</v>
@@ -7546,7 +7543,7 @@
         <v>12</v>
       </c>
       <c r="F182" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G182" s="9" t="s">
         <v>7</v>
@@ -7560,7 +7557,7 @@
         <v>28</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="D183" s="3" t="s">
         <v>208</v>
@@ -7569,7 +7566,7 @@
         <v>208</v>
       </c>
       <c r="F183" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G183" s="9" t="s">
         <v>209</v>
@@ -7583,7 +7580,7 @@
         <v>28</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="D184" s="3" t="s">
         <v>210</v>
@@ -7592,7 +7589,7 @@
         <v>210</v>
       </c>
       <c r="F184" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G184" s="9" t="s">
         <v>145</v>
@@ -7606,7 +7603,7 @@
         <v>28</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D185" s="3" t="s">
         <v>211</v>
@@ -7615,7 +7612,7 @@
         <v>211</v>
       </c>
       <c r="F185" s="9" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="G185" s="9" t="s">
         <v>183</v>
@@ -7629,7 +7626,7 @@
         <v>28</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D186" s="3" t="s">
         <v>212</v>
@@ -7638,7 +7635,7 @@
         <v>213</v>
       </c>
       <c r="F186" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G186" s="9" t="s">
         <v>38</v>
@@ -7652,16 +7649,16 @@
         <v>28</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D187" s="3" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E187" s="6" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="F187" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G187" s="9"/>
     </row>
@@ -7673,16 +7670,16 @@
         <v>28</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E188" s="3" t="s">
         <v>214</v>
       </c>
       <c r="F188" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G188" s="9"/>
     </row>
@@ -7694,16 +7691,16 @@
         <v>28</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E189" s="3" t="s">
         <v>215</v>
       </c>
       <c r="F189" s="9" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G189" s="9"/>
     </row>
@@ -7715,16 +7712,16 @@
         <v>28</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="D190" s="3" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="E190" s="3" t="s">
         <v>216</v>
       </c>
       <c r="F190" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G190" s="9"/>
     </row>
@@ -7762,7 +7759,7 @@
         <v>218</v>
       </c>
       <c r="D192" s="3" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E192" s="3" t="s">
         <v>219</v>
@@ -7804,7 +7801,7 @@
         <v>218</v>
       </c>
       <c r="D194" s="3" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E194" s="3" t="s">
         <v>221</v>
@@ -7825,7 +7822,7 @@
         <v>218</v>
       </c>
       <c r="D195" s="3" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E195" s="3" t="s">
         <v>222</v>
@@ -7846,7 +7843,7 @@
         <v>218</v>
       </c>
       <c r="D196" s="3" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="E196" s="3" t="s">
         <v>223</v>
@@ -7864,13 +7861,13 @@
         <v>2</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D197" s="3" t="s">
         <v>224</v>
       </c>
       <c r="E197" s="6" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F197" s="9" t="s">
         <v>40</v>
@@ -7885,13 +7882,13 @@
         <v>2</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>224</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F198" s="9" t="s">
         <v>40</v>
@@ -7906,13 +7903,13 @@
         <v>2</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D199" s="3" t="s">
         <v>224</v>
       </c>
       <c r="E199" s="3" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F199" s="9" t="s">
         <v>40</v>
@@ -7927,7 +7924,7 @@
         <v>2</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>224</v>
@@ -8038,13 +8035,13 @@
         <v>2</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="D205" s="3" t="s">
         <v>233</v>
       </c>
       <c r="E205" s="3" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="F205" s="9" t="s">
         <v>40</v>
@@ -8061,13 +8058,13 @@
         <v>2</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="D206" s="3" t="s">
         <v>233</v>
       </c>
       <c r="E206" s="3" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="F206" s="9" t="s">
         <v>40</v>
@@ -8084,13 +8081,13 @@
         <v>2</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="D207" s="3" t="s">
         <v>233</v>
       </c>
       <c r="E207" s="3" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="F207" s="9" t="s">
         <v>40</v>
@@ -8139,7 +8136,7 @@
         <v>238</v>
       </c>
       <c r="F209" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G209" s="9"/>
     </row>
@@ -8160,7 +8157,7 @@
         <v>239</v>
       </c>
       <c r="F210" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G210" s="9"/>
     </row>
@@ -8172,13 +8169,13 @@
         <v>112</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D211" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E211" s="6" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F211" s="9" t="s">
         <v>34</v>
@@ -8193,7 +8190,7 @@
         <v>112</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D212" s="3" t="s">
         <v>78</v>
@@ -8214,7 +8211,7 @@
         <v>112</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D213" s="3" t="s">
         <v>78</v>
@@ -8241,7 +8238,7 @@
         <v>241</v>
       </c>
       <c r="E214" s="6" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F214" s="9" t="s">
         <v>40</v>
@@ -8287,7 +8284,7 @@
         <v>243</v>
       </c>
       <c r="E216" s="6" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="F216" s="9" t="s">
         <v>4</v>
@@ -8330,7 +8327,7 @@
         <v>731</v>
       </c>
       <c r="D218" s="3" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E218" s="3" t="s">
         <v>245</v>
@@ -8351,7 +8348,7 @@
         <v>731</v>
       </c>
       <c r="D219" s="3" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="E219" s="3" t="s">
         <v>246</v>
@@ -8378,7 +8375,7 @@
         <v>247</v>
       </c>
       <c r="F220" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G220" s="9"/>
     </row>
@@ -8399,7 +8396,7 @@
         <v>248</v>
       </c>
       <c r="F221" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G221" s="9"/>
     </row>
@@ -8500,7 +8497,7 @@
         <v>800</v>
       </c>
       <c r="D226" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="E226" s="3" t="s">
         <v>251</v>
@@ -8572,7 +8569,7 @@
         <v>244</v>
       </c>
       <c r="E229" s="3" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="F229" s="9" t="s">
         <v>40</v>
@@ -8589,7 +8586,7 @@
         <v>35</v>
       </c>
       <c r="C230" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D230" s="3" t="s">
         <v>255</v>
@@ -8618,7 +8615,7 @@
         <v>78</v>
       </c>
       <c r="E231" s="6" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="F231" s="9" t="s">
         <v>10</v>
@@ -8660,7 +8657,7 @@
         <v>78</v>
       </c>
       <c r="E233" s="3" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="F233" s="9" t="s">
         <v>10</v>
@@ -8849,10 +8846,10 @@
         <v>148</v>
       </c>
       <c r="C242" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D242" s="3" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="E242" s="3" t="s">
         <v>264</v>
@@ -9040,10 +9037,10 @@
         <v>77</v>
       </c>
       <c r="C251" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D251" s="3" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="E251" s="3" t="s">
         <v>273</v>
@@ -9063,10 +9060,10 @@
         <v>77</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D252" s="3" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="E252" s="3" t="s">
         <v>275</v>
@@ -9086,10 +9083,10 @@
         <v>77</v>
       </c>
       <c r="C253" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D253" s="3" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="E253" s="3" t="s">
         <v>276</v>
@@ -9109,10 +9106,10 @@
         <v>77</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D254" s="3" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="E254" s="3" t="s">
         <v>277</v>
@@ -9155,7 +9152,7 @@
         <v>77</v>
       </c>
       <c r="C256" s="3" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="D256" s="3" t="s">
         <v>280</v>
@@ -9524,13 +9521,13 @@
         <v>807</v>
       </c>
       <c r="D272" s="3" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E272" s="3" t="s">
         <v>290</v>
       </c>
       <c r="F272" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G272" s="9" t="s">
         <v>183</v>
@@ -9547,13 +9544,13 @@
         <v>807</v>
       </c>
       <c r="D273" s="3" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E273" s="3" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="F273" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G273" s="9" t="s">
         <v>183</v>
@@ -9570,13 +9567,13 @@
         <v>807</v>
       </c>
       <c r="D274" s="3" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E274" s="3" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="F274" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G274" s="9" t="s">
         <v>183</v>
@@ -9593,13 +9590,13 @@
         <v>807</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="E275" s="3" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F275" s="9" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G275" s="9" t="s">
         <v>183</v>
@@ -9681,7 +9678,7 @@
         <v>218</v>
       </c>
       <c r="D279" s="3" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E279" s="3" t="s">
         <v>293</v>
@@ -10055,7 +10052,7 @@
         <v>305</v>
       </c>
       <c r="F295" s="9" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G295" s="9"/>
     </row>
@@ -10076,7 +10073,7 @@
         <v>306</v>
       </c>
       <c r="F296" s="9" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="G296" s="9"/>
     </row>
@@ -10139,7 +10136,7 @@
         <v>308</v>
       </c>
       <c r="F299" s="9" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="G299" s="9"/>
     </row>
@@ -10160,7 +10157,7 @@
         <v>309</v>
       </c>
       <c r="F300" s="9" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="G300" s="9"/>
     </row>
@@ -10181,7 +10178,7 @@
         <v>310</v>
       </c>
       <c r="F301" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G301" s="9"/>
     </row>
@@ -10202,7 +10199,7 @@
         <v>311</v>
       </c>
       <c r="F302" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G302" s="9"/>
     </row>
@@ -10223,7 +10220,7 @@
         <v>130</v>
       </c>
       <c r="F303" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G303" s="9"/>
     </row>
@@ -10244,7 +10241,7 @@
         <v>297</v>
       </c>
       <c r="F304" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G304" s="9"/>
     </row>
@@ -10262,7 +10259,7 @@
         <v>312</v>
       </c>
       <c r="E305" s="6" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F305" s="9" t="s">
         <v>66</v>
@@ -10370,7 +10367,7 @@
         <v>130</v>
       </c>
       <c r="F310" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G310" s="9"/>
     </row>
@@ -10391,7 +10388,7 @@
         <v>301</v>
       </c>
       <c r="F311" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G311" s="9"/>
     </row>
@@ -10412,7 +10409,7 @@
         <v>297</v>
       </c>
       <c r="F312" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G312" s="9"/>
     </row>
@@ -10433,7 +10430,7 @@
         <v>296</v>
       </c>
       <c r="F313" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G313" s="9"/>
     </row>
@@ -10496,7 +10493,7 @@
         <v>130</v>
       </c>
       <c r="F316" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G316" s="9"/>
     </row>
@@ -10517,7 +10514,7 @@
         <v>297</v>
       </c>
       <c r="F317" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G317" s="9"/>
     </row>
@@ -10538,7 +10535,7 @@
         <v>296</v>
       </c>
       <c r="F318" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G318" s="9"/>
     </row>
@@ -10622,7 +10619,7 @@
         <v>130</v>
       </c>
       <c r="F322" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G322" s="9"/>
     </row>
@@ -10643,7 +10640,7 @@
         <v>296</v>
       </c>
       <c r="F323" s="9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G323" s="9"/>
     </row>
@@ -10664,7 +10661,7 @@
         <v>313</v>
       </c>
       <c r="F324" s="9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G324" s="9"/>
     </row>
@@ -10685,7 +10682,7 @@
         <v>314</v>
       </c>
       <c r="F325" s="9" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="G325" s="9"/>
     </row>
@@ -10790,7 +10787,7 @@
         <v>130</v>
       </c>
       <c r="F330" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G330" s="9"/>
     </row>
@@ -10811,7 +10808,7 @@
         <v>296</v>
       </c>
       <c r="F331" s="9" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G331" s="9"/>
     </row>
@@ -10832,7 +10829,7 @@
         <v>130</v>
       </c>
       <c r="F332" s="9" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="G332" s="9"/>
     </row>
@@ -10871,7 +10868,7 @@
         <v>661</v>
       </c>
       <c r="E334" s="6" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="F334" s="9" t="s">
         <v>399</v>
@@ -10941,7 +10938,7 @@
         <v>130</v>
       </c>
       <c r="F337" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G337" s="9" t="s">
         <v>302</v>
@@ -10964,7 +10961,7 @@
         <v>296</v>
       </c>
       <c r="F338" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G338" s="9" t="s">
         <v>302</v>
@@ -10987,7 +10984,7 @@
         <v>297</v>
       </c>
       <c r="F339" s="9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G339" s="9" t="s">
         <v>302</v>
@@ -11033,7 +11030,7 @@
         <v>296</v>
       </c>
       <c r="F341" s="9" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="G341" s="9" t="s">
         <v>302</v>
@@ -11056,7 +11053,7 @@
         <v>296</v>
       </c>
       <c r="F342" s="9" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="G342" s="9" t="s">
         <v>302</v>
@@ -11079,7 +11076,7 @@
         <v>130</v>
       </c>
       <c r="F343" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G343" s="9" t="s">
         <v>302</v>
@@ -11102,7 +11099,7 @@
         <v>297</v>
       </c>
       <c r="F344" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G344" s="9" t="s">
         <v>302</v>
@@ -11125,7 +11122,7 @@
         <v>296</v>
       </c>
       <c r="F345" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G345" s="9" t="s">
         <v>302</v>
@@ -11283,7 +11280,7 @@
         <v>134</v>
       </c>
       <c r="E352" s="3" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="F352" s="9" t="s">
         <v>324</v>
@@ -11306,7 +11303,7 @@
         <v>134</v>
       </c>
       <c r="E353" s="3" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F353" s="9" t="s">
         <v>325</v>
@@ -11332,7 +11329,7 @@
         <v>326</v>
       </c>
       <c r="F354" s="9" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="G354" s="9" t="s">
         <v>183</v>
@@ -11355,7 +11352,7 @@
         <v>327</v>
       </c>
       <c r="F355" s="9" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="G355" s="9" t="s">
         <v>183</v>
@@ -11378,7 +11375,7 @@
         <v>328</v>
       </c>
       <c r="F356" s="9" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="G356" s="9" t="s">
         <v>183</v>
@@ -11424,7 +11421,7 @@
         <v>320</v>
       </c>
       <c r="F358" s="9" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="G358" s="9" t="s">
         <v>183</v>
@@ -12028,7 +12025,7 @@
         <v>134</v>
       </c>
       <c r="E385" s="3" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F385" s="9" t="s">
         <v>40</v>
@@ -12051,7 +12048,7 @@
         <v>134</v>
       </c>
       <c r="E386" s="3" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F386" s="9" t="s">
         <v>40</v>
@@ -12238,7 +12235,7 @@
         <v>351</v>
       </c>
       <c r="F394" s="9" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="G394" s="9" t="s">
         <v>7</v>
@@ -12307,7 +12304,7 @@
         <v>351</v>
       </c>
       <c r="F397" s="9" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="G397" s="9" t="s">
         <v>7</v>
@@ -12376,7 +12373,7 @@
         <v>168</v>
       </c>
       <c r="F400" s="9" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="G400" s="9" t="s">
         <v>170</v>
@@ -12413,13 +12410,13 @@
         <v>112</v>
       </c>
       <c r="C402" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D402" s="3" t="s">
         <v>358</v>
       </c>
       <c r="E402" s="4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F402" s="9" t="s">
         <v>101</v>
@@ -12434,7 +12431,7 @@
         <v>112</v>
       </c>
       <c r="C403" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D403" s="3" t="s">
         <v>358</v>
@@ -12464,7 +12461,7 @@
         <v>360</v>
       </c>
       <c r="F404" s="9" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="G404" s="9" t="s">
         <v>183</v>
@@ -12478,13 +12475,13 @@
         <v>112</v>
       </c>
       <c r="C405" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D405" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E405" s="4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F405" s="9" t="s">
         <v>101</v>
@@ -12524,7 +12521,7 @@
         <v>112</v>
       </c>
       <c r="C407" s="3" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D407" s="3" t="s">
         <v>78</v>
@@ -12547,7 +12544,7 @@
         <v>789</v>
       </c>
       <c r="C408" s="4" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="D408" s="3" t="s">
         <v>362</v>
@@ -12576,7 +12573,7 @@
         <v>364</v>
       </c>
       <c r="E409" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F409" s="9" t="s">
         <v>40</v>
@@ -12681,7 +12678,7 @@
         <v>358</v>
       </c>
       <c r="E414" s="4" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="F414" s="9" t="s">
         <v>40</v>
@@ -12761,13 +12758,13 @@
         <v>112</v>
       </c>
       <c r="C418" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D418" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E418" s="8" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F418" s="9" t="s">
         <v>4</v>
@@ -12784,13 +12781,13 @@
         <v>112</v>
       </c>
       <c r="C419" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D419" s="3" t="s">
         <v>373</v>
       </c>
       <c r="E419" s="8" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F419" s="9" t="s">
         <v>40</v>
@@ -12805,7 +12802,7 @@
         <v>112</v>
       </c>
       <c r="C420" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D420" s="3" t="s">
         <v>373</v>
@@ -12814,7 +12811,7 @@
         <v>374</v>
       </c>
       <c r="F420" s="9" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G420" s="9"/>
     </row>
@@ -12826,7 +12823,7 @@
         <v>112</v>
       </c>
       <c r="C421" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D421" s="3" t="s">
         <v>268</v>
@@ -12847,13 +12844,13 @@
         <v>112</v>
       </c>
       <c r="C422" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D422" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E422" s="4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F422" s="9" t="s">
         <v>4</v>
@@ -12868,7 +12865,7 @@
         <v>112</v>
       </c>
       <c r="C423" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D423" s="3" t="s">
         <v>78</v>
@@ -12889,7 +12886,7 @@
         <v>112</v>
       </c>
       <c r="C424" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D424" s="3" t="s">
         <v>78</v>
@@ -12898,7 +12895,7 @@
         <v>376</v>
       </c>
       <c r="F424" s="9" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="G424" s="9"/>
     </row>
@@ -12910,7 +12907,7 @@
         <v>112</v>
       </c>
       <c r="C425" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D425" s="3" t="s">
         <v>377</v>
@@ -12933,7 +12930,7 @@
         <v>112</v>
       </c>
       <c r="C426" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D426" s="3" t="s">
         <v>78</v>
@@ -12956,7 +12953,7 @@
         <v>112</v>
       </c>
       <c r="C427" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D427" s="3" t="s">
         <v>78</v>
@@ -12979,7 +12976,7 @@
         <v>112</v>
       </c>
       <c r="C428" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D428" s="3" t="s">
         <v>78</v>
@@ -13002,13 +12999,13 @@
         <v>112</v>
       </c>
       <c r="C429" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D429" s="3" t="s">
         <v>78</v>
       </c>
       <c r="E429" s="4" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F429" s="9" t="s">
         <v>101</v>
@@ -13186,7 +13183,7 @@
         <v>148</v>
       </c>
       <c r="C437" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D437" s="3" t="s">
         <v>386</v>
@@ -13301,7 +13298,7 @@
         <v>148</v>
       </c>
       <c r="C442" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D442" s="3" t="s">
         <v>386</v>
@@ -13324,7 +13321,7 @@
         <v>112</v>
       </c>
       <c r="C443" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D443" s="3" t="s">
         <v>397</v>
@@ -13560,7 +13557,7 @@
         <v>416</v>
       </c>
       <c r="E453" s="6" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="F453" s="9" t="s">
         <v>30</v>
@@ -13738,7 +13735,7 @@
         <v>35</v>
       </c>
       <c r="C461" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D461" s="3" t="s">
         <v>428</v>
@@ -13761,7 +13758,7 @@
         <v>35</v>
       </c>
       <c r="C462" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D462" s="3" t="s">
         <v>428</v>
@@ -13784,7 +13781,7 @@
         <v>35</v>
       </c>
       <c r="C463" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D463" s="3" t="s">
         <v>428</v>
@@ -13830,7 +13827,7 @@
         <v>35</v>
       </c>
       <c r="C465" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D465" s="3" t="s">
         <v>428</v>
@@ -13853,13 +13850,13 @@
         <v>148</v>
       </c>
       <c r="C466" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D466" s="3" t="s">
         <v>431</v>
       </c>
       <c r="E466" s="3" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="F466" s="9" t="s">
         <v>40</v>
@@ -13899,7 +13896,7 @@
         <v>112</v>
       </c>
       <c r="C468" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D468" s="3" t="s">
         <v>397</v>
@@ -13945,7 +13942,7 @@
         <v>2</v>
       </c>
       <c r="C470" s="4" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="D470" s="3" t="s">
         <v>436</v>
@@ -14083,7 +14080,7 @@
         <v>789</v>
       </c>
       <c r="C476" s="4" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="D476" s="3" t="s">
         <v>445</v>
@@ -14135,7 +14132,7 @@
         <v>452</v>
       </c>
       <c r="E478" s="3" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="F478" s="9" t="s">
         <v>66</v>
@@ -14158,7 +14155,7 @@
         <v>452</v>
       </c>
       <c r="E479" s="3" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="F479" s="9" t="s">
         <v>66</v>
@@ -14290,7 +14287,7 @@
         <v>112</v>
       </c>
       <c r="C485" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D485" s="3" t="s">
         <v>78</v>
@@ -14336,7 +14333,7 @@
         <v>112</v>
       </c>
       <c r="C487" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D487" s="3" t="s">
         <v>78</v>
@@ -14635,7 +14632,7 @@
         <v>112</v>
       </c>
       <c r="C500" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D500" s="3" t="s">
         <v>397</v>
@@ -14658,7 +14655,7 @@
         <v>112</v>
       </c>
       <c r="C501" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D501" s="3" t="s">
         <v>397</v>
@@ -14773,7 +14770,7 @@
         <v>28</v>
       </c>
       <c r="C506" s="4" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="D506" s="3" t="s">
         <v>484</v>
@@ -14796,7 +14793,7 @@
         <v>28</v>
       </c>
       <c r="C507" s="4" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="D507" s="3" t="s">
         <v>484</v>
@@ -14819,7 +14816,7 @@
         <v>112</v>
       </c>
       <c r="C508" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D508" s="3" t="s">
         <v>78</v>
@@ -14874,7 +14871,7 @@
         <v>488</v>
       </c>
       <c r="F510" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G510" s="9" t="s">
         <v>7</v>
@@ -14911,7 +14908,7 @@
         <v>28</v>
       </c>
       <c r="C512" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D512" s="3" t="s">
         <v>489</v>
@@ -15032,7 +15029,7 @@
         <v>495</v>
       </c>
       <c r="E517" s="3" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F517" s="9" t="s">
         <v>4</v>
@@ -15055,7 +15052,7 @@
         <v>495</v>
       </c>
       <c r="E518" s="3" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F518" s="9" t="s">
         <v>4</v>
@@ -15147,13 +15144,13 @@
         <v>500</v>
       </c>
       <c r="E522" s="3" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="F522" s="9" t="s">
         <v>90</v>
       </c>
       <c r="G522" s="9" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="523" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -15233,13 +15230,13 @@
         <v>112</v>
       </c>
       <c r="C526" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D526" s="3" t="s">
         <v>503</v>
       </c>
       <c r="E526" s="3" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="F526" s="9" t="s">
         <v>47</v>
@@ -15279,7 +15276,7 @@
         <v>112</v>
       </c>
       <c r="C528" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D528" s="3" t="s">
         <v>47</v>
@@ -15348,7 +15345,7 @@
         <v>148</v>
       </c>
       <c r="C531" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D531" s="3" t="s">
         <v>510</v>
@@ -15394,7 +15391,7 @@
         <v>28</v>
       </c>
       <c r="C533" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D533" s="3" t="s">
         <v>250</v>
@@ -15443,10 +15440,10 @@
         <v>403</v>
       </c>
       <c r="D535" s="3" t="s">
-        <v>815</v>
+        <v>934</v>
       </c>
       <c r="E535" s="3" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F535" s="9" t="s">
         <v>516</v>
@@ -15486,7 +15483,7 @@
         <v>28</v>
       </c>
       <c r="C537" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D537" s="3" t="s">
         <v>517</v>
@@ -15601,7 +15598,7 @@
         <v>28</v>
       </c>
       <c r="C542" s="7" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D542" s="3" t="s">
         <v>418</v>
@@ -15670,7 +15667,7 @@
         <v>112</v>
       </c>
       <c r="C545" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D545" s="3" t="s">
         <v>397</v>
@@ -15739,7 +15736,7 @@
         <v>77</v>
       </c>
       <c r="C548" s="4" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D548" s="3" t="s">
         <v>529</v>
@@ -15877,7 +15874,7 @@
         <v>2</v>
       </c>
       <c r="C554" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D554" s="3" t="s">
         <v>418</v>
@@ -15900,7 +15897,7 @@
         <v>2</v>
       </c>
       <c r="C555" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D555" s="3" t="s">
         <v>418</v>
@@ -15946,7 +15943,7 @@
         <v>112</v>
       </c>
       <c r="C557" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D557" s="3" t="s">
         <v>397</v>
@@ -15992,7 +15989,7 @@
         <v>112</v>
       </c>
       <c r="C559" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D559" s="3" t="s">
         <v>397</v>
@@ -16015,7 +16012,7 @@
         <v>28</v>
       </c>
       <c r="C560" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D560" s="3" t="s">
         <v>250</v>
@@ -16107,7 +16104,7 @@
         <v>112</v>
       </c>
       <c r="C564" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D564" s="3" t="s">
         <v>397</v>
@@ -16153,7 +16150,7 @@
         <v>112</v>
       </c>
       <c r="C566" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D566" s="3" t="s">
         <v>397</v>
@@ -16369,7 +16366,7 @@
         <v>238</v>
       </c>
       <c r="F575" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G575" s="9" t="s">
         <v>7</v>
@@ -16383,7 +16380,7 @@
         <v>112</v>
       </c>
       <c r="C576" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D576" s="3" t="s">
         <v>399</v>
@@ -16429,7 +16426,7 @@
         <v>549</v>
       </c>
       <c r="C578" s="4" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D578" s="3" t="s">
         <v>1</v>
@@ -16452,7 +16449,7 @@
         <v>549</v>
       </c>
       <c r="C579" s="4" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D579" s="3" t="s">
         <v>1</v>
@@ -16475,7 +16472,7 @@
         <v>549</v>
       </c>
       <c r="C580" s="4" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D580" s="3" t="s">
         <v>1</v>
@@ -17056,10 +17053,10 @@
         <v>130</v>
       </c>
       <c r="E605" s="3" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F605" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G605" s="9" t="s">
         <v>391</v>
@@ -17079,10 +17076,10 @@
         <v>130</v>
       </c>
       <c r="E606" s="3" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F606" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G606" s="9" t="s">
         <v>391</v>
@@ -17102,10 +17099,10 @@
         <v>130</v>
       </c>
       <c r="E607" s="3" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F607" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G607" s="9" t="s">
         <v>391</v>
@@ -17148,7 +17145,7 @@
         <v>495</v>
       </c>
       <c r="E609" s="3" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="F609" s="9" t="s">
         <v>4</v>
@@ -17194,7 +17191,7 @@
         <v>495</v>
       </c>
       <c r="E611" s="3" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="F611" s="9" t="s">
         <v>4</v>
@@ -17441,7 +17438,7 @@
         <v>77</v>
       </c>
       <c r="C622" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D622" s="3" t="s">
         <v>512</v>
@@ -17464,7 +17461,7 @@
         <v>148</v>
       </c>
       <c r="C623" s="4" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D623" s="3" t="s">
         <v>431</v>
@@ -17487,7 +17484,7 @@
         <v>35</v>
       </c>
       <c r="C624" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D624" s="3" t="s">
         <v>592</v>
@@ -17510,7 +17507,7 @@
         <v>35</v>
       </c>
       <c r="C625" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D625" s="3" t="s">
         <v>592</v>
@@ -17556,7 +17553,7 @@
         <v>77</v>
       </c>
       <c r="C627" s="4" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="D627" s="3" t="s">
         <v>596</v>
@@ -17648,7 +17645,7 @@
         <v>77</v>
       </c>
       <c r="C631" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D631" s="3" t="s">
         <v>599</v>
@@ -17671,7 +17668,7 @@
         <v>77</v>
       </c>
       <c r="C632" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D632" s="3" t="s">
         <v>599</v>
@@ -17763,7 +17760,7 @@
         <v>77</v>
       </c>
       <c r="C636" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D636" s="3" t="s">
         <v>599</v>
@@ -17786,7 +17783,7 @@
         <v>77</v>
       </c>
       <c r="C637" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D637" s="3" t="s">
         <v>599</v>
@@ -17809,7 +17806,7 @@
         <v>77</v>
       </c>
       <c r="C638" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D638" s="3" t="s">
         <v>599</v>
@@ -17832,7 +17829,7 @@
         <v>77</v>
       </c>
       <c r="C639" s="4" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D639" s="3" t="s">
         <v>599</v>
@@ -18005,7 +18002,7 @@
         <v>4</v>
       </c>
       <c r="G646" s="9" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="647" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -18016,7 +18013,7 @@
         <v>28</v>
       </c>
       <c r="C647" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="D647" s="3" t="s">
         <v>250</v>
@@ -18361,7 +18358,7 @@
         <v>77</v>
       </c>
       <c r="C662" s="4" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D662" s="3" t="s">
         <v>99</v>
@@ -18407,7 +18404,7 @@
         <v>112</v>
       </c>
       <c r="C664" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D664" s="3" t="s">
         <v>397</v>
@@ -18430,7 +18427,7 @@
         <v>112</v>
       </c>
       <c r="C665" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D665" s="3" t="s">
         <v>397</v>
@@ -18453,13 +18450,13 @@
         <v>112</v>
       </c>
       <c r="C666" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D666" s="3" t="s">
         <v>397</v>
       </c>
       <c r="E666" s="3" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F666" s="9" t="s">
         <v>40</v>
@@ -18476,7 +18473,7 @@
         <v>112</v>
       </c>
       <c r="C667" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D667" s="3" t="s">
         <v>397</v>
@@ -18499,13 +18496,13 @@
         <v>112</v>
       </c>
       <c r="C668" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D668" s="3" t="s">
         <v>397</v>
       </c>
       <c r="E668" s="3" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F668" s="9" t="s">
         <v>53</v>
@@ -18522,7 +18519,7 @@
         <v>112</v>
       </c>
       <c r="C669" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D669" s="3" t="s">
         <v>397</v>
@@ -18545,7 +18542,7 @@
         <v>112</v>
       </c>
       <c r="C670" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D670" s="3" t="s">
         <v>113</v>
@@ -18568,7 +18565,7 @@
         <v>112</v>
       </c>
       <c r="C671" s="7" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="D671" s="3" t="s">
         <v>113</v>
@@ -18670,7 +18667,7 @@
         <v>90</v>
       </c>
       <c r="G675" s="9" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
     </row>
     <row r="676" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -18693,7 +18690,7 @@
         <v>4</v>
       </c>
       <c r="G676" s="9" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="677" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -18727,7 +18724,7 @@
         <v>112</v>
       </c>
       <c r="C678" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D678" s="3" t="s">
         <v>656</v>
@@ -18762,7 +18759,7 @@
         <v>109</v>
       </c>
       <c r="G679" s="9" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="680" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -18865,7 +18862,7 @@
         <v>112</v>
       </c>
       <c r="C684" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="D684" s="3" t="s">
         <v>658</v>
@@ -18888,7 +18885,7 @@
         <v>112</v>
       </c>
       <c r="C685" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="D685" s="3" t="s">
         <v>658</v>
@@ -18911,7 +18908,7 @@
         <v>112</v>
       </c>
       <c r="C686" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="D686" s="3" t="s">
         <v>658</v>
@@ -19124,7 +19121,7 @@
         <v>661</v>
       </c>
       <c r="E695" s="3" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="F695" s="9" t="s">
         <v>40</v>
@@ -19199,7 +19196,7 @@
         <v>16</v>
       </c>
       <c r="G698" s="9" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="699" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -19233,7 +19230,7 @@
         <v>2</v>
       </c>
       <c r="C700" s="4" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="D700" s="3" t="s">
         <v>674</v>
@@ -19325,7 +19322,7 @@
         <v>28</v>
       </c>
       <c r="C704" s="7" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D704" s="3" t="s">
         <v>674</v>
@@ -19495,7 +19492,7 @@
         <v>687</v>
       </c>
       <c r="F711" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G711" s="9" t="s">
         <v>7</v>
@@ -19518,7 +19515,7 @@
         <v>688</v>
       </c>
       <c r="F712" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G712" s="9" t="s">
         <v>7</v>
@@ -19716,7 +19713,7 @@
         <v>77</v>
       </c>
       <c r="C721" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D721" s="3"/>
       <c r="E721" s="3" t="s">
@@ -19737,7 +19734,7 @@
         <v>77</v>
       </c>
       <c r="C722" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D722" s="7"/>
       <c r="E722" s="3" t="s">
@@ -19758,7 +19755,7 @@
         <v>77</v>
       </c>
       <c r="C723" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D723" s="7"/>
       <c r="E723" s="3" t="s">
@@ -19779,7 +19776,7 @@
         <v>77</v>
       </c>
       <c r="C724" s="4" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D724" s="7"/>
       <c r="E724" s="3" t="s">
@@ -19858,7 +19855,7 @@
         <v>4</v>
       </c>
       <c r="G727" s="9" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="728" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -19961,7 +19958,7 @@
         <v>2</v>
       </c>
       <c r="C732" s="4" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="D732" s="3" t="s">
         <v>90</v>
@@ -19984,7 +19981,7 @@
         <v>2</v>
       </c>
       <c r="C733" s="4" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="D733" s="3" t="s">
         <v>90</v>
@@ -20076,7 +20073,7 @@
         <v>77</v>
       </c>
       <c r="C737" s="4" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="D737" s="3" t="s">
         <v>721</v>
@@ -20108,7 +20105,7 @@
         <v>724</v>
       </c>
       <c r="F738" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G738" s="9" t="s">
         <v>7</v>
@@ -20131,7 +20128,7 @@
         <v>724</v>
       </c>
       <c r="F739" s="9" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="G739" s="9" t="s">
         <v>7</v>
@@ -20145,7 +20142,7 @@
         <v>129</v>
       </c>
       <c r="C740" s="4" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="D740" s="3" t="s">
         <v>726</v>
@@ -20191,7 +20188,7 @@
         <v>35</v>
       </c>
       <c r="C742" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D742" s="3" t="s">
         <v>428</v>
@@ -20214,7 +20211,7 @@
         <v>35</v>
       </c>
       <c r="C743" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D743" s="3" t="s">
         <v>428</v>
@@ -20237,7 +20234,7 @@
         <v>35</v>
       </c>
       <c r="C744" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D744" s="3" t="s">
         <v>428</v>
@@ -20260,7 +20257,7 @@
         <v>35</v>
       </c>
       <c r="C745" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="D745" s="3" t="s">
         <v>428</v>
@@ -20479,7 +20476,7 @@
         <v>40</v>
       </c>
       <c r="G754" s="9" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="755" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -20519,7 +20516,7 @@
         <v>478</v>
       </c>
       <c r="E756" s="3" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="F756" s="9" t="s">
         <v>4</v>
@@ -20542,7 +20539,7 @@
         <v>478</v>
       </c>
       <c r="E757" s="3" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="F757" s="9" t="s">
         <v>4</v>
@@ -20565,7 +20562,7 @@
         <v>478</v>
       </c>
       <c r="E758" s="3" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="F758" s="9" t="s">
         <v>4</v>
@@ -20588,7 +20585,7 @@
         <v>478</v>
       </c>
       <c r="E759" s="3" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="F759" s="9" t="s">
         <v>4</v>
@@ -20611,7 +20608,7 @@
         <v>478</v>
       </c>
       <c r="E760" s="3" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="F760" s="9" t="s">
         <v>4</v>
@@ -20634,7 +20631,7 @@
         <v>478</v>
       </c>
       <c r="E761" s="3" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F761" s="9" t="s">
         <v>4</v>
@@ -20657,7 +20654,7 @@
         <v>478</v>
       </c>
       <c r="E762" s="3" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F762" s="9" t="s">
         <v>4</v>
@@ -20680,7 +20677,7 @@
         <v>478</v>
       </c>
       <c r="E763" s="3" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F763" s="9" t="s">
         <v>4</v>
@@ -20881,7 +20878,7 @@
         <v>77</v>
       </c>
       <c r="C772" s="4" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D772" s="3" t="s">
         <v>763</v>
@@ -20939,7 +20936,7 @@
         <v>53</v>
       </c>
       <c r="G774" s="9" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="775" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -20962,7 +20959,7 @@
         <v>53</v>
       </c>
       <c r="G775" s="9" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="776" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -20985,7 +20982,7 @@
         <v>670</v>
       </c>
       <c r="G776" s="9" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="777" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -20996,7 +20993,7 @@
         <v>77</v>
       </c>
       <c r="C777" s="3" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="D777" s="3" t="s">
         <v>768</v>
@@ -21054,7 +21051,7 @@
         <v>4</v>
       </c>
       <c r="G779" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="780" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21077,7 +21074,7 @@
         <v>47</v>
       </c>
       <c r="G780" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="781" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21100,7 +21097,7 @@
         <v>40</v>
       </c>
       <c r="G781" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="782" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21123,7 +21120,7 @@
         <v>53</v>
       </c>
       <c r="G782" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="783" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21146,7 +21143,7 @@
         <v>66</v>
       </c>
       <c r="G783" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="784" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21169,7 +21166,7 @@
         <v>298</v>
       </c>
       <c r="G784" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="785" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21192,7 +21189,7 @@
         <v>429</v>
       </c>
       <c r="G785" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="786" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21215,7 +21212,7 @@
         <v>10</v>
       </c>
       <c r="G786" s="9" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="787" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21238,7 +21235,7 @@
         <v>53</v>
       </c>
       <c r="G787" s="9" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="788" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21261,7 +21258,7 @@
         <v>354</v>
       </c>
       <c r="G788" s="9" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="789" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
@@ -21295,7 +21292,7 @@
         <v>112</v>
       </c>
       <c r="C790" s="4" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D790" s="3" t="s">
         <v>147</v>
@@ -21513,7 +21510,7 @@
         <v>77</v>
       </c>
       <c r="C800" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D800" s="3" t="s">
         <v>780</v>
@@ -21522,7 +21519,7 @@
         <v>780</v>
       </c>
       <c r="F800" s="9" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="G800" s="9" t="s">
         <v>430</v>
@@ -21536,7 +21533,7 @@
         <v>77</v>
       </c>
       <c r="C801" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D801" s="3" t="s">
         <v>780</v>
@@ -21545,7 +21542,7 @@
         <v>780</v>
       </c>
       <c r="F801" s="9" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="G801" s="9" t="s">
         <v>38</v>
@@ -21559,7 +21556,7 @@
         <v>77</v>
       </c>
       <c r="C802" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D802" s="3" t="s">
         <v>780</v>
@@ -21582,7 +21579,7 @@
         <v>77</v>
       </c>
       <c r="C803" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D803" s="3" t="s">
         <v>780</v>
@@ -21605,7 +21602,7 @@
         <v>77</v>
       </c>
       <c r="C804" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D804" s="3" t="s">
         <v>780</v>
@@ -21628,7 +21625,7 @@
         <v>77</v>
       </c>
       <c r="C805" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D805" s="3" t="s">
         <v>780</v>
@@ -21651,7 +21648,7 @@
         <v>77</v>
       </c>
       <c r="C806" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D806" s="3" t="s">
         <v>780</v>
@@ -21674,7 +21671,7 @@
         <v>77</v>
       </c>
       <c r="C807" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D807" s="3" t="s">
         <v>780</v>
@@ -21697,7 +21694,7 @@
         <v>77</v>
       </c>
       <c r="C808" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D808" s="3" t="s">
         <v>780</v>
@@ -21720,7 +21717,7 @@
         <v>77</v>
       </c>
       <c r="C809" s="3" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D809" s="3" t="s">
         <v>780</v>
@@ -21766,7 +21763,7 @@
         <v>810</v>
       </c>
       <c r="C811" s="4" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D811" s="4" t="s">
         <v>783</v>
@@ -21789,7 +21786,7 @@
         <v>810</v>
       </c>
       <c r="C812" s="3" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="D812" s="3" t="s">
         <v>786</v>
@@ -21812,7 +21809,7 @@
         <v>789</v>
       </c>
       <c r="C813" s="8" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="D813" s="3" t="s">
         <v>788</v>

</xml_diff>